<commit_message>
Sync P002 concise Excel sheet with linked agent-topic details
</commit_message>
<xml_diff>
--- a/papers/P002/P002_工程复现问题清单_v1.xlsx
+++ b/papers/P002/P002_工程复现问题清单_v1.xlsx
@@ -9,7 +9,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <fonts count="3">
+  <fonts count="2">
     <font>
       <sz val="11"/>
       <name val="Aptos"/>
@@ -19,12 +19,6 @@
       <sz val="11"/>
       <name val="Aptos"/>
       <color rgb="FFFFFFFF"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <name val="Aptos"/>
-      <u/>
-      <color rgb="FF0563C1"/>
     </font>
   </fonts>
   <fills count="4">
@@ -59,18 +53,15 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
+      <alignment wrapText="1" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
+      <alignment wrapText="1" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
+      <alignment wrapText="1" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -82,14 +73,14 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:C14"/>
-  <sheetFormatPr defaultRowHeight="25"/>
+  <sheetFormatPr defaultRowHeight="24"/>
   <cols>
     <col min="1" max="1" width="23" customWidth="1"/>
-    <col min="2" max="2" width="54" customWidth="1"/>
-    <col min="3" max="3" width="95" customWidth="1"/>
+    <col min="2" max="2" width="51" customWidth="1"/>
+    <col min="3" max="3" width="92" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" ht="40" customHeight="1">
+    <row r="1" ht="36" customHeight="1">
       <c r="A1" t="inlineStr" s="1">
         <is>
           <t xml:space="preserve">主题</t>
@@ -106,7 +97,7 @@
         </is>
       </c>
     </row>
-    <row r="2" ht="155" customHeight="1">
+    <row r="2" ht="100" customHeight="1">
       <c r="A2" t="inlineStr" s="0">
         <is>
           <t xml:space="preserve">金融专题Agent</t>
@@ -114,16 +105,16 @@
       </c>
       <c r="B2" t="inlineStr" s="0">
         <is>
-          <t xml:space="preserve">七层21类金融Agent分别有哪些？如何实现？</t>
-        </is>
-      </c>
-      <c r="C2" t="inlineStr" s="3">
-        <is>
-          <t xml:space="preserve">I市场周期/波动状态(2)；II尾部风险/崩盘预警(2)；III流动性/订单失衡/量价协同/成交量结构(4)；IV趋势/反转/区间波动/滞后响应/波动非对称(5)；V回撤/分形(2)；VI状态门控/稳定性(2)；VII K线形态/创造性设计/因子组合/羊群效应(4)。每类有专门金融任务Prompt，不是21个微调模型。详见作者21个原始Prompt：https://github.com/uwFengyuan/CogAlpha_Prompt/tree/main/prompts/seven_level_agent_hierarchy</t>
-        </is>
-      </c>
-    </row>
-    <row r="3" ht="93" customHeight="1">
+          <t xml:space="preserve">21个金融专题Agent怎样分工，具体靠什么实现？</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">作者按7个金融研究层级定义21种专业角色。每种角色以独立的研究任务Intro和因子设计Guidance，搭配统一的代码与输出模板组成Prompt；并不是21个分别微调的模型。具体分类及每份原始Prompt，点击查看：https://github.com/epshoron/JXwork/blob/main/papers/P002/P002_AGENT_TOPICS.md</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="86" customHeight="1">
       <c r="A3" t="inlineStr" s="2">
         <is>
           <t xml:space="preserve">模型与Agent实现</t>
@@ -140,7 +131,7 @@
         </is>
       </c>
     </row>
-    <row r="4" ht="93" customHeight="1">
+    <row r="4" ht="86" customHeight="1">
       <c r="A4" t="inlineStr" s="0">
         <is>
           <t xml:space="preserve">五种Guidance</t>
@@ -157,7 +148,7 @@
         </is>
       </c>
     </row>
-    <row r="5" ht="93" customHeight="1">
+    <row r="5" ht="86" customHeight="1">
       <c r="A5" t="inlineStr" s="2">
         <is>
           <t xml:space="preserve">代码输入输出</t>
@@ -174,7 +165,7 @@
         </is>
       </c>
     </row>
-    <row r="6" ht="93" customHeight="1">
+    <row r="6" ht="86" customHeight="1">
       <c r="A6" t="inlineStr" s="0">
         <is>
           <t xml:space="preserve">质量检查</t>
@@ -191,7 +182,7 @@
         </is>
       </c>
     </row>
-    <row r="7" ht="93" customHeight="1">
+    <row r="7" ht="86" customHeight="1">
       <c r="A7" t="inlineStr" s="2">
         <is>
           <t xml:space="preserve">预测评分</t>
@@ -208,7 +199,7 @@
         </is>
       </c>
     </row>
-    <row r="8" ht="93" customHeight="1">
+    <row r="8" ht="86" customHeight="1">
       <c r="A8" t="inlineStr" s="0">
         <is>
           <t xml:space="preserve">保留规则</t>
@@ -225,7 +216,7 @@
         </is>
       </c>
     </row>
-    <row r="9" ht="93" customHeight="1">
+    <row r="9" ht="86" customHeight="1">
       <c r="A9" t="inlineStr" s="2">
         <is>
           <t xml:space="preserve">反馈再生成</t>
@@ -242,7 +233,7 @@
         </is>
       </c>
     </row>
-    <row r="10" ht="93" customHeight="1">
+    <row r="10" ht="86" customHeight="1">
       <c r="A10" t="inlineStr" s="0">
         <is>
           <t xml:space="preserve">显式与隐式遗传</t>
@@ -259,7 +250,7 @@
         </is>
       </c>
     </row>
-    <row r="11" ht="93" customHeight="1">
+    <row r="11" ht="86" customHeight="1">
       <c r="A11" t="inlineStr" s="2">
         <is>
           <t xml:space="preserve">Mutation与Crossover</t>
@@ -276,7 +267,7 @@
         </is>
       </c>
     </row>
-    <row r="12" ht="93" customHeight="1">
+    <row r="12" ht="86" customHeight="1">
       <c r="A12" t="inlineStr" s="0">
         <is>
           <t xml:space="preserve">两路衔接</t>
@@ -293,7 +284,7 @@
         </is>
       </c>
     </row>
-    <row r="13" ht="93" customHeight="1">
+    <row r="13" ht="86" customHeight="1">
       <c r="A13" t="inlineStr" s="2">
         <is>
           <t xml:space="preserve">循环控制</t>
@@ -310,7 +301,7 @@
         </is>
       </c>
     </row>
-    <row r="14" ht="93" customHeight="1">
+    <row r="14" ht="86" customHeight="1">
       <c r="A14" t="inlineStr" s="0">
         <is>
           <t xml:space="preserve">公开实现与复现</t>
@@ -330,7 +321,7 @@
   </sheetData>
   <autoFilter ref="A1:C14"/>
   <hyperlinks>
-    <hyperlink ref="C2" r:id="rId1" tooltip="点击打开作者21个Agent Prompt目录"/>
+    <hyperlink ref="C2" r:id="rId1" tooltip="点击阅读七层21个专题及原始Prompt"/>
   </hyperlinks>
 </worksheet>
 </file>
</xml_diff>